<commit_message>
update: modify Monthly Back-up Monitoring Sheet for improved functionality
</commit_message>
<xml_diff>
--- a/forms/F-MIS-06 Monthly Back-up Monitoring Sheet(1).xlsx
+++ b/forms/F-MIS-06 Monthly Back-up Monitoring Sheet(1).xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MIS FORMS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\wamp64\www\MISDB\forms\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{766AE1B6-B94F-4AFF-A591-709194F98EA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96BCF8D2-E5AF-40D7-B0AD-57ED78AEE51D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2424,16 +2424,36 @@
       <c r="C5" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D5" s="4"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4"/>
-      <c r="K5" s="3"/>
-      <c r="L5" s="3"/>
-      <c r="M5" s="3"/>
+      <c r="D5" s="4">
+        <v>46029</v>
+      </c>
+      <c r="E5" s="4">
+        <v>46057</v>
+      </c>
+      <c r="F5" s="4">
+        <v>46090</v>
+      </c>
+      <c r="G5" s="4">
+        <v>46119</v>
+      </c>
+      <c r="H5" s="4">
+        <v>46152</v>
+      </c>
+      <c r="I5" s="4">
+        <v>46187</v>
+      </c>
+      <c r="J5" s="4">
+        <v>46208</v>
+      </c>
+      <c r="K5" s="4">
+        <v>46245</v>
+      </c>
+      <c r="L5" s="4">
+        <v>46280</v>
+      </c>
+      <c r="M5" s="4">
+        <v>46301</v>
+      </c>
       <c r="N5" s="3"/>
       <c r="O5" s="3"/>
     </row>

</xml_diff>